<commit_message>
Agrego variable de grado de urbanización a personas
</commit_message>
<xml_diff>
--- a/data-raw/xlsx/tabla_advertencias.xlsx
+++ b/data-raw/xlsx/tabla_advertencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fernando_gallegos\Proyectos\odsa.eusilc\data-raw\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067359E0-1FE3-4BC2-ACA9-BD2BF23715A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E75B8C8E-4213-4692-8236-3C770A75C95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="197">
   <si>
     <t>id_advertencia</t>
   </si>
@@ -584,6 +584,33 @@
   </si>
   <si>
     <t>El paquete deja los ingresos ausentes</t>
+  </si>
+  <si>
+    <t>urbanizacion_de_pre2021</t>
+  </si>
+  <si>
+    <t>DB100</t>
+  </si>
+  <si>
+    <t>Alemania no reporta el grado de urbanización</t>
+  </si>
+  <si>
+    <t>pi07 queda completamente ausente</t>
+  </si>
+  <si>
+    <t>El paquete conserva DB100 como ausente</t>
+  </si>
+  <si>
+    <t>urbanizacion_de_post2021</t>
+  </si>
+  <si>
+    <t>Alemania unifica los códigos 1 y 2 en 1</t>
+  </si>
+  <si>
+    <t>pi07 no se ve afectada</t>
+  </si>
+  <si>
+    <t>El paquete utiliza la recodificación armonizada pi07</t>
   </si>
 </sst>
 </file>
@@ -936,9 +963,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3868,6 +3896,82 @@
         <v>182</v>
       </c>
     </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>188</v>
+      </c>
+      <c r="B78">
+        <v>2015</v>
+      </c>
+      <c r="C78">
+        <v>2020</v>
+      </c>
+      <c r="D78" t="s">
+        <v>20</v>
+      </c>
+      <c r="E78" t="s">
+        <v>12</v>
+      </c>
+      <c r="F78" t="s">
+        <v>13</v>
+      </c>
+      <c r="G78" t="s">
+        <v>189</v>
+      </c>
+      <c r="H78" t="s">
+        <v>47</v>
+      </c>
+      <c r="I78" t="s">
+        <v>190</v>
+      </c>
+      <c r="J78" t="s">
+        <v>191</v>
+      </c>
+      <c r="K78" t="s">
+        <v>192</v>
+      </c>
+      <c r="L78" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>193</v>
+      </c>
+      <c r="B79">
+        <v>2021</v>
+      </c>
+      <c r="C79">
+        <v>2025</v>
+      </c>
+      <c r="D79" t="s">
+        <v>20</v>
+      </c>
+      <c r="E79" t="s">
+        <v>12</v>
+      </c>
+      <c r="F79" t="s">
+        <v>13</v>
+      </c>
+      <c r="G79" t="s">
+        <v>189</v>
+      </c>
+      <c r="H79" t="s">
+        <v>15</v>
+      </c>
+      <c r="I79" t="s">
+        <v>194</v>
+      </c>
+      <c r="J79" t="s">
+        <v>195</v>
+      </c>
+      <c r="K79" t="s">
+        <v>196</v>
+      </c>
+      <c r="L79" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrego urbanización a hogares
</commit_message>
<xml_diff>
--- a/data-raw/xlsx/tabla_advertencias.xlsx
+++ b/data-raw/xlsx/tabla_advertencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fernando_gallegos\Proyectos\odsa.eusilc\data-raw\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E75B8C8E-4213-4692-8236-3C770A75C95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D26ED3-553B-41CB-B37D-EAA3F509D5C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="199">
   <si>
     <t>id_advertencia</t>
   </si>
@@ -611,6 +611,12 @@
   </si>
   <si>
     <t>El paquete utiliza la recodificación armonizada pi07</t>
+  </si>
+  <si>
+    <t>hi07 queda completamente ausente</t>
+  </si>
+  <si>
+    <t>hi07 no se ve afectada</t>
   </si>
 </sst>
 </file>
@@ -963,7 +969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
@@ -3972,6 +3978,82 @@
         <v>19</v>
       </c>
     </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>188</v>
+      </c>
+      <c r="B80">
+        <v>2015</v>
+      </c>
+      <c r="C80">
+        <v>2020</v>
+      </c>
+      <c r="D80" t="s">
+        <v>20</v>
+      </c>
+      <c r="E80" t="s">
+        <v>108</v>
+      </c>
+      <c r="F80" t="s">
+        <v>13</v>
+      </c>
+      <c r="G80" t="s">
+        <v>189</v>
+      </c>
+      <c r="H80" t="s">
+        <v>47</v>
+      </c>
+      <c r="I80" t="s">
+        <v>190</v>
+      </c>
+      <c r="J80" t="s">
+        <v>197</v>
+      </c>
+      <c r="K80" t="s">
+        <v>192</v>
+      </c>
+      <c r="L80" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>193</v>
+      </c>
+      <c r="B81">
+        <v>2021</v>
+      </c>
+      <c r="C81">
+        <v>2025</v>
+      </c>
+      <c r="D81" t="s">
+        <v>20</v>
+      </c>
+      <c r="E81" t="s">
+        <v>108</v>
+      </c>
+      <c r="F81" t="s">
+        <v>13</v>
+      </c>
+      <c r="G81" t="s">
+        <v>189</v>
+      </c>
+      <c r="H81" t="s">
+        <v>15</v>
+      </c>
+      <c r="I81" t="s">
+        <v>194</v>
+      </c>
+      <c r="J81" t="s">
+        <v>198</v>
+      </c>
+      <c r="K81" t="s">
+        <v>196</v>
+      </c>
+      <c r="L81" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>